<commit_message>
Update all reports with LBMA daily gold data and new best Dyn 2x3x (G0.5)
- Gold data: LBMA AM fix daily (14,720 rows, 1968-2026)
  replaces monthly interpolation that underestimated volatility
- Best Dyn 2x3x changes: G0.6 → G0.5 (equal Gold/Bond split)
- New metrics: CAGR 31.40% (was 30.67%), Sharpe 1.297, WF 0.885
- DH Dynamic CAGR25+ also updated: CAGR 25.60% (was 25.23%)
- Regenerated: YEARLY_RETURNS_REPORT.md, Excel v2, all CSVs

https://claude.ai/code/session_01AnaE6CMbDeeFYPv77Xs27G
</commit_message>
<xml_diff>
--- a/YEARLY_RETURNS_7STRATEGIES_v2.xlsx
+++ b/YEARLY_RETURNS_7STRATEGIES_v2.xlsx
@@ -655,7 +655,8 @@
       <c r="B12" s="7" t="inlineStr">
         <is>
           <t>A2+Gold2x(2036)
-+Bond3x(TMF) *</t>
++Bond3x(TMF)
+G0.5/B0.5 *</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -702,10 +703,10 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.3067</v>
+        <v>0.314</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>0.2523</v>
+        <v>0.256</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>0.2919</v>
@@ -779,10 +780,10 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>0.3067</v>
+        <v>0.314</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>0.2523</v>
+        <v>0.256</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>0.2919</v>
@@ -807,10 +808,10 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>0.3183228580325856</v>
+        <v>0.3222312438988297</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>0.2724172919543411</v>
+        <v>0.2940435269869324</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>0.2618094703587007</v>
@@ -835,10 +836,10 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>1.443456425602937</v>
+        <v>1.458597218825991</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>1.35875267377596</v>
+        <v>1.383801197237958</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>2.213621488235486</v>
@@ -863,10 +864,10 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>-0.1658267964277036</v>
+        <v>-0.1893881862108775</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>-0.1265113932269826</v>
+        <v>-0.1249745778198378</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>-0.2507263406918773</v>
@@ -891,10 +892,10 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>0.3447427503819926</v>
+        <v>0.346792385305604</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>0.2943119212659813</v>
+        <v>0.2969375686511043</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>0.4445165596702268</v>
@@ -919,7 +920,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>44</v>
@@ -947,7 +948,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>9</v>
@@ -1022,10 +1023,10 @@
         <v>1974</v>
       </c>
       <c r="B26" s="15" t="n">
-        <v>0.242921445227865</v>
+        <v>0.3132099472063998</v>
       </c>
       <c r="C26" s="15" t="n">
-        <v>0.1114174568433617</v>
+        <v>0.1789676773008375</v>
       </c>
       <c r="D26" s="15" t="n">
         <v>0</v>
@@ -1048,10 +1049,10 @@
         <v>1975</v>
       </c>
       <c r="B27" s="15" t="n">
-        <v>0.008547798158128561</v>
+        <v>0.01727581347492713</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>0.05206122966712612</v>
+        <v>0.05031396824835688</v>
       </c>
       <c r="D27" s="15" t="n">
         <v>0.1440942281560682</v>
@@ -1074,10 +1075,10 @@
         <v>1976</v>
       </c>
       <c r="B28" s="15" t="n">
-        <v>0.604997528306032</v>
+        <v>0.6353928732511757</v>
       </c>
       <c r="C28" s="15" t="n">
-        <v>0.5082880300514738</v>
+        <v>0.516642230941776</v>
       </c>
       <c r="D28" s="15" t="n">
         <v>0.6825772668916013</v>
@@ -1100,10 +1101,10 @@
         <v>1977</v>
       </c>
       <c r="B29" s="15" t="n">
-        <v>0.1118054164536504</v>
+        <v>0.08155741702160825</v>
       </c>
       <c r="C29" s="15" t="n">
-        <v>0.06948039762331115</v>
+        <v>0.06002464807589147</v>
       </c>
       <c r="D29" s="15" t="n">
         <v>0.02580031066730371</v>
@@ -1126,10 +1127,10 @@
         <v>1978</v>
       </c>
       <c r="B30" s="15" t="n">
-        <v>0.7427865699836</v>
+        <v>0.7351448460749148</v>
       </c>
       <c r="C30" s="15" t="n">
-        <v>0.643696279585937</v>
+        <v>0.6608915241067269</v>
       </c>
       <c r="D30" s="15" t="n">
         <v>0.6105822073840994</v>
@@ -1152,10 +1153,10 @@
         <v>1979</v>
       </c>
       <c r="B31" s="15" t="n">
-        <v>0.7834662523433351</v>
+        <v>0.5542349941672404</v>
       </c>
       <c r="C31" s="15" t="n">
-        <v>0.4623950050341969</v>
+        <v>0.4085557146220759</v>
       </c>
       <c r="D31" s="15" t="n">
         <v>0.2066930732204824</v>
@@ -1178,10 +1179,10 @@
         <v>1980</v>
       </c>
       <c r="B32" s="15" t="n">
-        <v>0.6820108743699965</v>
+        <v>0.9069004752197545</v>
       </c>
       <c r="C32" s="15" t="n">
-        <v>0.5648183306317341</v>
+        <v>0.6714283927458016</v>
       </c>
       <c r="D32" s="15" t="n">
         <v>0.7724834783120376</v>
@@ -1204,10 +1205,10 @@
         <v>1981</v>
       </c>
       <c r="B33" s="16" t="n">
-        <v>-0.1375230157871715</v>
+        <v>-0.1014674643710533</v>
       </c>
       <c r="C33" s="16" t="n">
-        <v>-0.09593607940668493</v>
+        <v>-0.08906404129941992</v>
       </c>
       <c r="D33" s="16" t="n">
         <v>-0.07309568724104054</v>
@@ -1230,10 +1231,10 @@
         <v>1982</v>
       </c>
       <c r="B34" s="15" t="n">
-        <v>1.012662664487005</v>
+        <v>1.041687247164218</v>
       </c>
       <c r="C34" s="15" t="n">
-        <v>0.6545944354376791</v>
+        <v>0.6527439329702192</v>
       </c>
       <c r="D34" s="15" t="n">
         <v>0.8239838912198256</v>
@@ -1256,10 +1257,10 @@
         <v>1983</v>
       </c>
       <c r="B35" s="15" t="n">
-        <v>0.3869266186683169</v>
+        <v>0.4612860353332411</v>
       </c>
       <c r="C35" s="15" t="n">
-        <v>0.4151055239708994</v>
+        <v>0.4646755675966653</v>
       </c>
       <c r="D35" s="15" t="n">
         <v>0.7252954023677592</v>
@@ -1281,11 +1282,11 @@
       <c r="A36" s="14" t="n">
         <v>1984</v>
       </c>
-      <c r="B36" s="16" t="n">
-        <v>-0.0325811458591746</v>
+      <c r="B36" s="15" t="n">
+        <v>0.009310212218380354</v>
       </c>
       <c r="C36" s="16" t="n">
-        <v>-0.02294568495468274</v>
+        <v>-0.02057025950817748</v>
       </c>
       <c r="D36" s="16" t="n">
         <v>-0.04681722901282615</v>
@@ -1308,10 +1309,10 @@
         <v>1985</v>
       </c>
       <c r="B37" s="15" t="n">
-        <v>0.8539083473232839</v>
+        <v>0.8662463089406358</v>
       </c>
       <c r="C37" s="15" t="n">
-        <v>0.6646476312475865</v>
+        <v>0.6512984127288913</v>
       </c>
       <c r="D37" s="15" t="n">
         <v>0.8240836545452386</v>
@@ -1334,10 +1335,10 @@
         <v>1986</v>
       </c>
       <c r="B38" s="15" t="n">
-        <v>0.5051154345315405</v>
+        <v>0.5644737031337769</v>
       </c>
       <c r="C38" s="15" t="n">
-        <v>0.3487203422238021</v>
+        <v>0.3797486198217453</v>
       </c>
       <c r="D38" s="15" t="n">
         <v>0.2886556068116617</v>
@@ -1360,10 +1361,10 @@
         <v>1987</v>
       </c>
       <c r="B39" s="15" t="n">
-        <v>0.3183228580325856</v>
+        <v>0.3589252048099247</v>
       </c>
       <c r="C39" s="15" t="n">
-        <v>0.2231196878436484</v>
+        <v>0.2486943763664331</v>
       </c>
       <c r="D39" s="15" t="n">
         <v>0.1323394141692327</v>
@@ -1386,10 +1387,10 @@
         <v>1988</v>
       </c>
       <c r="B40" s="16" t="n">
-        <v>-0.07879994261077761</v>
+        <v>-0.05462255252670401</v>
       </c>
       <c r="C40" s="16" t="n">
-        <v>-0.05509604365913301</v>
+        <v>-0.05319787080906102</v>
       </c>
       <c r="D40" s="16" t="n">
         <v>-0.04009659602281069</v>
@@ -1412,10 +1413,10 @@
         <v>1989</v>
       </c>
       <c r="B41" s="15" t="n">
-        <v>0.488152843174662</v>
+        <v>0.482985365422673</v>
       </c>
       <c r="C41" s="15" t="n">
-        <v>0.3940104536936824</v>
+        <v>0.3838162380382304</v>
       </c>
       <c r="D41" s="15" t="n">
         <v>0.4316231498727383</v>
@@ -1438,10 +1439,10 @@
         <v>1990</v>
       </c>
       <c r="B42" s="16" t="n">
-        <v>-0.05772937700206848</v>
+        <v>-0.002136376955472307</v>
       </c>
       <c r="C42" s="16" t="n">
-        <v>-0.04780037580080377</v>
+        <v>-0.02566985215077144</v>
       </c>
       <c r="D42" s="16" t="n">
         <v>-0.1217451426862551</v>
@@ -1464,10 +1465,10 @@
         <v>1991</v>
       </c>
       <c r="B43" s="15" t="n">
-        <v>0.6242267743452914</v>
+        <v>0.6640257544707306</v>
       </c>
       <c r="C43" s="15" t="n">
-        <v>0.5500517979734378</v>
+        <v>0.5474582187969528</v>
       </c>
       <c r="D43" s="15" t="n">
         <v>0.8652924905122881</v>
@@ -1490,10 +1491,10 @@
         <v>1992</v>
       </c>
       <c r="B44" s="15" t="n">
-        <v>0.3258247288155418</v>
+        <v>0.3463642560275897</v>
       </c>
       <c r="C44" s="15" t="n">
-        <v>0.2971087862665462</v>
+        <v>0.3025985971121623</v>
       </c>
       <c r="D44" s="15" t="n">
         <v>0.4557061958415698</v>
@@ -1516,10 +1517,10 @@
         <v>1993</v>
       </c>
       <c r="B45" s="15" t="n">
-        <v>0.1482704182829548</v>
+        <v>0.125615309109653</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>0.07458021464130438</v>
+        <v>0.06841604603396512</v>
       </c>
       <c r="D45" s="15" t="n">
         <v>0.01614640026870684</v>
@@ -1542,10 +1543,10 @@
         <v>1994</v>
       </c>
       <c r="B46" s="16" t="n">
-        <v>-0.02322609864946268</v>
+        <v>-0.04984760226536888</v>
       </c>
       <c r="C46" s="16" t="n">
-        <v>-0.007032439301531079</v>
+        <v>-0.01865095653083615</v>
       </c>
       <c r="D46" s="16" t="n">
         <v>-0.008687537033379766</v>
@@ -1568,10 +1569,10 @@
         <v>1995</v>
       </c>
       <c r="B47" s="15" t="n">
-        <v>0.8836888293488753</v>
+        <v>0.8646093021164095</v>
       </c>
       <c r="C47" s="15" t="n">
-        <v>0.7234453956502551</v>
+        <v>0.7126310917582263</v>
       </c>
       <c r="D47" s="15" t="n">
         <v>1.119553473211065</v>
@@ -1594,10 +1595,10 @@
         <v>1996</v>
       </c>
       <c r="B48" s="15" t="n">
-        <v>0.2801830157974612</v>
+        <v>0.3222312438988297</v>
       </c>
       <c r="C48" s="15" t="n">
-        <v>0.2724172919543411</v>
+        <v>0.2940435269869324</v>
       </c>
       <c r="D48" s="15" t="n">
         <v>0.4338587518724679</v>
@@ -1620,10 +1621,10 @@
         <v>1997</v>
       </c>
       <c r="B49" s="15" t="n">
-        <v>0.6253652978171254</v>
+        <v>0.6537901433646289</v>
       </c>
       <c r="C49" s="15" t="n">
-        <v>0.6173620694613529</v>
+        <v>0.6007668445169125</v>
       </c>
       <c r="D49" s="15" t="n">
         <v>0.9632474168757765</v>
@@ -1646,10 +1647,10 @@
         <v>1998</v>
       </c>
       <c r="B50" s="15" t="n">
-        <v>0.8198955566403892</v>
+        <v>0.8378986425559865</v>
       </c>
       <c r="C50" s="15" t="n">
-        <v>0.6924616869454528</v>
+        <v>0.6852559789963597</v>
       </c>
       <c r="D50" s="15" t="n">
         <v>0.8529744447456642</v>
@@ -1672,10 +1673,10 @@
         <v>1999</v>
       </c>
       <c r="B51" s="15" t="n">
-        <v>1.443456425602937</v>
+        <v>1.458597218825991</v>
       </c>
       <c r="C51" s="15" t="n">
-        <v>1.35875267377596</v>
+        <v>1.383801197237958</v>
       </c>
       <c r="D51" s="15" t="n">
         <v>2.213621488235486</v>
@@ -1698,10 +1699,10 @@
         <v>2000</v>
       </c>
       <c r="B52" s="15" t="n">
-        <v>0.0274392924396103</v>
+        <v>0.05978742290593764</v>
       </c>
       <c r="C52" s="15" t="n">
-        <v>0.002627304396334518</v>
+        <v>0.005751243859183353</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>-0.04451311860812989</v>
@@ -1724,10 +1725,10 @@
         <v>2001</v>
       </c>
       <c r="B53" s="15" t="n">
-        <v>0.0361024931228926</v>
+        <v>0.03557879783507722</v>
       </c>
       <c r="C53" s="15" t="n">
-        <v>0.01548503646299437</v>
+        <v>0.01551853014956595</v>
       </c>
       <c r="D53" s="15" t="n">
         <v>0</v>
@@ -1750,10 +1751,10 @@
         <v>2002</v>
       </c>
       <c r="B54" s="15" t="n">
-        <v>0.2214083408356808</v>
+        <v>0.2124739968172351</v>
       </c>
       <c r="C54" s="15" t="n">
-        <v>0.1026686845682971</v>
+        <v>0.09938581660957624</v>
       </c>
       <c r="D54" s="15" t="n">
         <v>0</v>
@@ -1776,10 +1777,10 @@
         <v>2003</v>
       </c>
       <c r="B55" s="15" t="n">
-        <v>0.7382907103181222</v>
+        <v>0.7465878787940814</v>
       </c>
       <c r="C55" s="15" t="n">
-        <v>0.6681870519649238</v>
+        <v>0.6742501683707264</v>
       </c>
       <c r="D55" s="15" t="n">
         <v>0.99277512546135</v>
@@ -1802,10 +1803,10 @@
         <v>2004</v>
       </c>
       <c r="B56" s="15" t="n">
-        <v>0.1404294241967385</v>
+        <v>0.1255544418776573</v>
       </c>
       <c r="C56" s="15" t="n">
-        <v>0.1082283529339987</v>
+        <v>0.09872296483766595</v>
       </c>
       <c r="D56" s="15" t="n">
         <v>0.06764548510048485</v>
@@ -1828,10 +1829,10 @@
         <v>2005</v>
       </c>
       <c r="B57" s="15" t="n">
-        <v>0.0568132532500627</v>
+        <v>0.05267012665770765</v>
       </c>
       <c r="C57" s="15" t="n">
-        <v>0.03032357837003397</v>
+        <v>0.03196683510048737</v>
       </c>
       <c r="D57" s="16" t="n">
         <v>-0.0121529109892613</v>
@@ -1854,10 +1855,10 @@
         <v>2006</v>
       </c>
       <c r="B58" s="15" t="n">
-        <v>0.4821302774804619</v>
+        <v>0.480747950140098</v>
       </c>
       <c r="C58" s="15" t="n">
-        <v>0.4075075854559312</v>
+        <v>0.4163473552781827</v>
       </c>
       <c r="D58" s="15" t="n">
         <v>0.5275268242666009</v>
@@ -1880,10 +1881,10 @@
         <v>2007</v>
       </c>
       <c r="B59" s="15" t="n">
-        <v>0.2618396330033279</v>
+        <v>0.2610741505926255</v>
       </c>
       <c r="C59" s="15" t="n">
-        <v>0.1796582690292347</v>
+        <v>0.1765326359969392</v>
       </c>
       <c r="D59" s="15" t="n">
         <v>0.1340851575566344</v>
@@ -1906,10 +1907,10 @@
         <v>2008</v>
       </c>
       <c r="B60" s="15" t="n">
-        <v>0.08366356167727297</v>
+        <v>0.1080826046359762</v>
       </c>
       <c r="C60" s="15" t="n">
-        <v>0.02704759742690022</v>
+        <v>0.02235702145282126</v>
       </c>
       <c r="D60" s="16" t="n">
         <v>-0.07947835675457104</v>
@@ -1932,10 +1933,10 @@
         <v>2009</v>
       </c>
       <c r="B61" s="15" t="n">
-        <v>0.4750052361018113</v>
+        <v>0.4506359720013779</v>
       </c>
       <c r="C61" s="15" t="n">
-        <v>0.4267548075148984</v>
+        <v>0.4341154834338856</v>
       </c>
       <c r="D61" s="15" t="n">
         <v>0.5432225225653364</v>
@@ -1958,10 +1959,10 @@
         <v>2010</v>
       </c>
       <c r="B62" s="15" t="n">
-        <v>0.4582668602220004</v>
+        <v>0.4389635179715665</v>
       </c>
       <c r="C62" s="15" t="n">
-        <v>0.3544635142269217</v>
+        <v>0.3509272293419368</v>
       </c>
       <c r="D62" s="15" t="n">
         <v>0.2618094703587007</v>
@@ -1984,10 +1985,10 @@
         <v>2011</v>
       </c>
       <c r="B63" s="16" t="n">
-        <v>-0.06153162536876033</v>
+        <v>-0.07776782974056951</v>
       </c>
       <c r="C63" s="16" t="n">
-        <v>-0.1265113932269826</v>
+        <v>-0.1249745778198378</v>
       </c>
       <c r="D63" s="16" t="n">
         <v>-0.2507263406918773</v>
@@ -2010,10 +2011,10 @@
         <v>2012</v>
       </c>
       <c r="B64" s="15" t="n">
-        <v>0.3505456429067679</v>
+        <v>0.339188066176333</v>
       </c>
       <c r="C64" s="15" t="n">
-        <v>0.3200129485359837</v>
+        <v>0.3138004120888904</v>
       </c>
       <c r="D64" s="15" t="n">
         <v>0.4132602164271597</v>
@@ -2036,10 +2037,10 @@
         <v>2013</v>
       </c>
       <c r="B65" s="15" t="n">
-        <v>0.2697290070162073</v>
+        <v>0.2720003757431892</v>
       </c>
       <c r="C65" s="15" t="n">
-        <v>0.3318676102978755</v>
+        <v>0.3250246737481635</v>
       </c>
       <c r="D65" s="15" t="n">
         <v>0.7666927557492802</v>
@@ -2062,10 +2063,10 @@
         <v>2014</v>
       </c>
       <c r="B66" s="15" t="n">
-        <v>0.04746700552497551</v>
+        <v>0.06512180542790125</v>
       </c>
       <c r="C66" s="15" t="n">
-        <v>0.0398356493645784</v>
+        <v>0.04280653738224038</v>
       </c>
       <c r="D66" s="15" t="n">
         <v>0.07898958587284111</v>
@@ -2088,10 +2089,10 @@
         <v>2015</v>
       </c>
       <c r="B67" s="16" t="n">
-        <v>-0.1408201115682326</v>
+        <v>-0.1316255191346717</v>
       </c>
       <c r="C67" s="16" t="n">
-        <v>-0.1151410709672913</v>
+        <v>-0.1179125357001342</v>
       </c>
       <c r="D67" s="16" t="n">
         <v>-0.1369020782663063</v>
@@ -2114,10 +2115,10 @@
         <v>2016</v>
       </c>
       <c r="B68" s="15" t="n">
-        <v>0.07063827889319141</v>
+        <v>0.06472304559697806</v>
       </c>
       <c r="C68" s="15" t="n">
-        <v>0.02233331962874807</v>
+        <v>0.02213275751369204</v>
       </c>
       <c r="D68" s="16" t="n">
         <v>-0.05227806871659989</v>
@@ -2140,10 +2141,10 @@
         <v>2017</v>
       </c>
       <c r="B69" s="15" t="n">
-        <v>0.374456854503777</v>
+        <v>0.3701881406799415</v>
       </c>
       <c r="C69" s="15" t="n">
-        <v>0.3329804758130857</v>
+        <v>0.3324149536454506</v>
       </c>
       <c r="D69" s="15" t="n">
         <v>0.4953903838713161</v>
@@ -2166,10 +2167,10 @@
         <v>2018</v>
       </c>
       <c r="B70" s="15" t="n">
-        <v>0.1254313179662778</v>
+        <v>0.1206933665000453</v>
       </c>
       <c r="C70" s="15" t="n">
-        <v>0.100598416988714</v>
+        <v>0.1008955049855376</v>
       </c>
       <c r="D70" s="15" t="n">
         <v>0.05952629287363354</v>
@@ -2192,10 +2193,10 @@
         <v>2019</v>
       </c>
       <c r="B71" s="15" t="n">
-        <v>0.4708301470455738</v>
+        <v>0.4849880594325257</v>
       </c>
       <c r="C71" s="15" t="n">
-        <v>0.3821679957955462</v>
+        <v>0.3908183801252634</v>
       </c>
       <c r="D71" s="15" t="n">
         <v>0.4761379368410685</v>
@@ -2218,10 +2219,10 @@
         <v>2020</v>
       </c>
       <c r="B72" s="15" t="n">
-        <v>0.7233293343613554</v>
+        <v>0.7149108814676733</v>
       </c>
       <c r="C72" s="15" t="n">
-        <v>0.6204657761335497</v>
+        <v>0.6069756316185102</v>
       </c>
       <c r="D72" s="15" t="n">
         <v>0.6848733699986262</v>
@@ -2244,10 +2245,10 @@
         <v>2021</v>
       </c>
       <c r="B73" s="15" t="n">
-        <v>0.273161822462945</v>
+        <v>0.260917822259463</v>
       </c>
       <c r="C73" s="15" t="n">
-        <v>0.2574752818710651</v>
+        <v>0.2534012945170965</v>
       </c>
       <c r="D73" s="15" t="n">
         <v>0.4037643767197108</v>
@@ -2270,10 +2271,10 @@
         <v>2022</v>
       </c>
       <c r="B74" s="16" t="n">
-        <v>-0.1658267964277036</v>
+        <v>-0.1893881862108775</v>
       </c>
       <c r="C74" s="16" t="n">
-        <v>-0.108779177738955</v>
+        <v>-0.1104256189913709</v>
       </c>
       <c r="D74" s="16" t="n">
         <v>-0.1176258515769151</v>
@@ -2296,10 +2297,10 @@
         <v>2023</v>
       </c>
       <c r="B75" s="15" t="n">
-        <v>0.4700657864357869</v>
+        <v>0.4777865835036594</v>
       </c>
       <c r="C75" s="15" t="n">
-        <v>0.4030314751076863</v>
+        <v>0.4044599213984292</v>
       </c>
       <c r="D75" s="15" t="n">
         <v>0.5138054298081998</v>
@@ -2322,10 +2323,10 @@
         <v>2024</v>
       </c>
       <c r="B76" s="15" t="n">
-        <v>0.3573064742164838</v>
+        <v>0.3064322405390476</v>
       </c>
       <c r="C76" s="15" t="n">
-        <v>0.2575531954636097</v>
+        <v>0.2394036158286319</v>
       </c>
       <c r="D76" s="15" t="n">
         <v>0.2605117095441229</v>
@@ -2348,10 +2349,10 @@
         <v>2025</v>
       </c>
       <c r="B77" s="15" t="n">
-        <v>0.5889643510474</v>
+        <v>0.5143878874195449</v>
       </c>
       <c r="C77" s="15" t="n">
-        <v>0.3714167118536076</v>
+        <v>0.3689810750056759</v>
       </c>
       <c r="D77" s="15" t="n">
         <v>0.2902467751719067</v>
@@ -2374,10 +2375,10 @@
         <v>2026</v>
       </c>
       <c r="B78" s="16" t="n">
-        <v>-0.1101643468644917</v>
+        <v>-0.09016501006217925</v>
       </c>
       <c r="C78" s="16" t="n">
-        <v>-0.08505296271368845</v>
+        <v>-0.07817656875216605</v>
       </c>
       <c r="D78" s="16" t="n">
         <v>-0.1118534403426848</v>
@@ -2451,10 +2452,10 @@
         </is>
       </c>
       <c r="B82" s="15" t="n">
-        <v>0.01426035346607812</v>
+        <v>0.0154828622773131</v>
       </c>
       <c r="C82" s="15" t="n">
-        <v>0.01727110073848115</v>
+        <v>0.01777651048502471</v>
       </c>
       <c r="D82" s="15" t="n">
         <v>0.02870472795491796</v>
@@ -2479,10 +2480,10 @@
         </is>
       </c>
       <c r="B83" s="16" t="n">
-        <v>-0.01096142249031296</v>
+        <v>-0.003326952619756351</v>
       </c>
       <c r="C83" s="15" t="n">
-        <v>0.0006755154592403829</v>
+        <v>0.004178500118459104</v>
       </c>
       <c r="D83" s="15" t="n">
         <v>0.01627755740598813</v>
@@ -2507,10 +2508,10 @@
         </is>
       </c>
       <c r="B84" s="16" t="n">
-        <v>-0.01674012446981188</v>
+        <v>-0.03060442456949775</v>
       </c>
       <c r="C84" s="16" t="n">
-        <v>-0.009659101653672232</v>
+        <v>-0.01783690359216039</v>
       </c>
       <c r="D84" s="16" t="n">
         <v>-0.003911718342873516</v>
@@ -2535,10 +2536,10 @@
         </is>
       </c>
       <c r="B85" s="15" t="n">
-        <v>0.05366895288463946</v>
+        <v>0.05959085807805131</v>
       </c>
       <c r="C85" s="15" t="n">
-        <v>0.04291060661675195</v>
+        <v>0.04771940019963217</v>
       </c>
       <c r="D85" s="15" t="n">
         <v>0.05882264681228633</v>
@@ -2563,10 +2564,10 @@
         </is>
       </c>
       <c r="B86" s="16" t="n">
-        <v>-0.005664615333201506</v>
+        <v>-0.01314947656592824</v>
       </c>
       <c r="C86" s="16" t="n">
-        <v>-0.02078705993265451</v>
+        <v>-0.02190051600533938</v>
       </c>
       <c r="D86" s="16" t="n">
         <v>-0.05934102256568385</v>
@@ -2591,10 +2592,10 @@
         </is>
       </c>
       <c r="B87" s="15" t="n">
-        <v>0.04477701209079354</v>
+        <v>0.05039521008148973</v>
       </c>
       <c r="C87" s="15" t="n">
-        <v>0.0508402108297985</v>
+        <v>0.05059347215296328</v>
       </c>
       <c r="D87" s="15" t="n">
         <v>0.09847653646198572</v>
@@ -2619,10 +2620,10 @@
         </is>
       </c>
       <c r="B88" s="15" t="n">
-        <v>0.0329373440961529</v>
+        <v>0.03628956797320115</v>
       </c>
       <c r="C88" s="15" t="n">
-        <v>0.02707784317183925</v>
+        <v>0.02936632825956797</v>
       </c>
       <c r="D88" s="15" t="n">
         <v>0.02953406508393664</v>
@@ -2647,10 +2648,10 @@
         </is>
       </c>
       <c r="B89" s="15" t="n">
-        <v>0.0891788650927763</v>
+        <v>0.08691247612789187</v>
       </c>
       <c r="C89" s="15" t="n">
-        <v>0.08486140230876416</v>
+        <v>0.08352500384301242</v>
       </c>
       <c r="D89" s="15" t="n">
         <v>0.1138726428444201</v>
@@ -2675,10 +2676,10 @@
         </is>
       </c>
       <c r="B90" s="16" t="n">
-        <v>-0.06983794938469423</v>
+        <v>-0.07698032378406461</v>
       </c>
       <c r="C90" s="16" t="n">
-        <v>-0.05953015197483048</v>
+        <v>-0.06365005238288446</v>
       </c>
       <c r="D90" s="16" t="n">
         <v>-0.07873542449358739</v>
@@ -2703,10 +2704,10 @@
         </is>
       </c>
       <c r="B91" s="15" t="n">
-        <v>0.07355448765676065</v>
+        <v>0.08019258039738573</v>
       </c>
       <c r="C91" s="15" t="n">
-        <v>0.06670936028154539</v>
+        <v>0.07255412179485909</v>
       </c>
       <c r="D91" s="15" t="n">
         <v>0.1023995407681799</v>
@@ -2731,10 +2732,10 @@
         </is>
       </c>
       <c r="B92" s="15" t="n">
-        <v>0.03872650527808452</v>
+        <v>0.04291554198686121</v>
       </c>
       <c r="C92" s="15" t="n">
-        <v>0.03475327067679035</v>
+        <v>0.03564907681180318</v>
       </c>
       <c r="D92" s="15" t="n">
         <v>0.04966229732321414</v>
@@ -2758,11 +2759,11 @@
           <t>2021-12</t>
         </is>
       </c>
-      <c r="B93" s="15" t="n">
-        <v>0.01049650519593626</v>
-      </c>
-      <c r="C93" s="15" t="n">
-        <v>0.004889809304654768</v>
+      <c r="B93" s="16" t="n">
+        <v>-0.0009640006009584701</v>
+      </c>
+      <c r="C93" s="16" t="n">
+        <v>-0.000226671660478294</v>
       </c>
       <c r="D93" s="15" t="n">
         <v>0.007854528742709199</v>
@@ -2787,10 +2788,10 @@
         </is>
       </c>
       <c r="B94" s="16" t="n">
-        <v>-0.09405515792165042</v>
+        <v>-0.09603094329819896</v>
       </c>
       <c r="C94" s="16" t="n">
-        <v>-0.08040486919679646</v>
+        <v>-0.07969544343951707</v>
       </c>
       <c r="D94" s="16" t="n">
         <v>-0.1036569453885952</v>
@@ -2815,10 +2816,10 @@
         </is>
       </c>
       <c r="B95" s="15" t="n">
-        <v>0.03419185989120654</v>
+        <v>0.02597767904654646</v>
       </c>
       <c r="C95" s="15" t="n">
-        <v>0.01425819180947197</v>
+        <v>0.0146426984076844</v>
       </c>
       <c r="D95" s="16" t="n">
         <v>-0.01558433025888284</v>
@@ -2843,10 +2844,10 @@
         </is>
       </c>
       <c r="B96" s="16" t="n">
-        <v>-0.01145735810291948</v>
+        <v>-0.03052001999902521</v>
       </c>
       <c r="C96" s="16" t="n">
-        <v>-0.000537321457946937</v>
+        <v>-0.00743744788288736</v>
       </c>
       <c r="D96" s="15" t="n">
         <v>0</v>
@@ -2871,10 +2872,10 @@
         </is>
       </c>
       <c r="B97" s="16" t="n">
-        <v>-0.03531033232634317</v>
+        <v>-0.03080761325180048</v>
       </c>
       <c r="C97" s="16" t="n">
-        <v>-0.01570721874534875</v>
+        <v>-0.0106898039721377</v>
       </c>
       <c r="D97" s="15" t="n">
         <v>0</v>
@@ -2899,10 +2900,10 @@
         </is>
       </c>
       <c r="B98" s="16" t="n">
-        <v>-0.02262171613322195</v>
+        <v>-0.0170490004003343</v>
       </c>
       <c r="C98" s="16" t="n">
-        <v>-0.009804300360304108</v>
+        <v>-0.00919801516331442</v>
       </c>
       <c r="D98" s="15" t="n">
         <v>0</v>
@@ -2927,10 +2928,10 @@
         </is>
       </c>
       <c r="B99" s="16" t="n">
-        <v>-0.01559204975596196</v>
+        <v>-0.01663426219641773</v>
       </c>
       <c r="C99" s="16" t="n">
-        <v>-0.007514203447170131</v>
+        <v>-0.008189855091831122</v>
       </c>
       <c r="D99" s="15" t="n">
         <v>0</v>
@@ -2955,10 +2956,10 @@
         </is>
       </c>
       <c r="B100" s="15" t="n">
-        <v>0.003862723217769703</v>
-      </c>
-      <c r="C100" s="15" t="n">
-        <v>0.0005135324426452921</v>
+        <v>0.00513393405336493</v>
+      </c>
+      <c r="C100" s="16" t="n">
+        <v>-0.002176763275356541</v>
       </c>
       <c r="D100" s="15" t="n">
         <v>0</v>
@@ -2983,10 +2984,10 @@
         </is>
       </c>
       <c r="B101" s="16" t="n">
-        <v>-0.03496027944661262</v>
+        <v>-0.03571992810124713</v>
       </c>
       <c r="C101" s="16" t="n">
-        <v>-0.01595564687619777</v>
+        <v>-0.01537208019691394</v>
       </c>
       <c r="D101" s="15" t="n">
         <v>0</v>
@@ -3011,10 +3012,10 @@
         </is>
       </c>
       <c r="B102" s="16" t="n">
-        <v>-0.0456169795179494</v>
+        <v>-0.04640475744301131</v>
       </c>
       <c r="C102" s="16" t="n">
-        <v>-0.02090362747411001</v>
+        <v>-0.01949216886109584</v>
       </c>
       <c r="D102" s="15" t="n">
         <v>0</v>
@@ -3039,10 +3040,10 @@
         </is>
       </c>
       <c r="B103" s="16" t="n">
-        <v>-0.02663060337373002</v>
+        <v>-0.02979690816882197</v>
       </c>
       <c r="C103" s="16" t="n">
-        <v>-0.01190490812420852</v>
+        <v>-0.01321328383038944</v>
       </c>
       <c r="D103" s="15" t="n">
         <v>0</v>
@@ -3067,10 +3068,10 @@
         </is>
       </c>
       <c r="B104" s="15" t="n">
-        <v>0.05624002907410874</v>
+        <v>0.06344720311181941</v>
       </c>
       <c r="C104" s="15" t="n">
-        <v>0.02630402121196851</v>
+        <v>0.03134286385031571</v>
       </c>
       <c r="D104" s="15" t="n">
         <v>0</v>
@@ -3095,10 +3096,10 @@
         </is>
       </c>
       <c r="B105" s="15" t="n">
-        <v>0.0208219492072117</v>
+        <v>0.009150363337427692</v>
       </c>
       <c r="C105" s="15" t="n">
-        <v>0.01103470878919155</v>
+        <v>0.006997950289512778</v>
       </c>
       <c r="D105" s="15" t="n">
         <v>0</v>
@@ -3123,10 +3124,10 @@
         </is>
       </c>
       <c r="B106" s="15" t="n">
-        <v>0.04833729184464519</v>
+        <v>0.04145954052092438</v>
       </c>
       <c r="C106" s="15" t="n">
-        <v>0.02297884319308841</v>
+        <v>0.02038586422494637</v>
       </c>
       <c r="D106" s="15" t="n">
         <v>0</v>
@@ -3151,10 +3152,10 @@
         </is>
       </c>
       <c r="B107" s="16" t="n">
-        <v>-0.1224734409818938</v>
+        <v>-0.1170862690584616</v>
       </c>
       <c r="C107" s="16" t="n">
-        <v>-0.1014442987829183</v>
+        <v>-0.09935459418440107</v>
       </c>
       <c r="D107" s="16" t="n">
         <v>-0.1157266207586112</v>
@@ -3179,10 +3180,10 @@
         </is>
       </c>
       <c r="B108" s="15" t="n">
-        <v>0.1893561535681869</v>
+        <v>0.1916797515431532</v>
       </c>
       <c r="C108" s="15" t="n">
-        <v>0.1644186202497524</v>
+        <v>0.1669381114116455</v>
       </c>
       <c r="D108" s="15" t="n">
         <v>0.1996534391125415</v>
@@ -3207,10 +3208,10 @@
         </is>
       </c>
       <c r="B109" s="16" t="n">
-        <v>-0.00093242924106196</v>
+        <v>-0.002544282078354332</v>
       </c>
       <c r="C109" s="16" t="n">
-        <v>-0.001935175157395829</v>
+        <v>-0.003014597075851499</v>
       </c>
       <c r="D109" s="16" t="n">
         <v>-0.004914450927922531</v>
@@ -3235,10 +3236,10 @@
         </is>
       </c>
       <c r="B110" s="15" t="n">
-        <v>0.08507667054182821</v>
+        <v>0.08541415913942618</v>
       </c>
       <c r="C110" s="15" t="n">
-        <v>0.08316140959853759</v>
+        <v>0.08336675062733301</v>
       </c>
       <c r="D110" s="15" t="n">
         <v>0.1239972063106549</v>
@@ -3263,10 +3264,10 @@
         </is>
       </c>
       <c r="B111" s="15" t="n">
-        <v>0.1482094705503747</v>
+        <v>0.1469465353608341</v>
       </c>
       <c r="C111" s="15" t="n">
-        <v>0.1419969294799481</v>
+        <v>0.1409560474140874</v>
       </c>
       <c r="D111" s="15" t="n">
         <v>0.2029825025661567</v>
@@ -3291,10 +3292,10 @@
         </is>
       </c>
       <c r="B112" s="15" t="n">
-        <v>0.1013998439986543</v>
+        <v>0.1004622729212468</v>
       </c>
       <c r="C112" s="15" t="n">
-        <v>0.0938253564983369</v>
+        <v>0.09420636263569149</v>
       </c>
       <c r="D112" s="15" t="n">
         <v>0.1206248216542256</v>
@@ -3319,10 +3320,10 @@
         </is>
       </c>
       <c r="B113" s="16" t="n">
-        <v>-0.1051469863771802</v>
+        <v>-0.1015767740488689</v>
       </c>
       <c r="C113" s="16" t="n">
-        <v>-0.09806447500905124</v>
+        <v>-0.09681209649150813</v>
       </c>
       <c r="D113" s="16" t="n">
         <v>-0.1202919463419843</v>
@@ -3347,10 +3348,10 @@
         </is>
       </c>
       <c r="B114" s="16" t="n">
-        <v>-0.08407839209688583</v>
+        <v>-0.0803872391532684</v>
       </c>
       <c r="C114" s="16" t="n">
-        <v>-0.06384645355920515</v>
+        <v>-0.06168684676849379</v>
       </c>
       <c r="D114" s="16" t="n">
         <v>-0.07897416124054268</v>
@@ -3375,10 +3376,10 @@
         </is>
       </c>
       <c r="B115" s="16" t="n">
-        <v>-0.04566644142845244</v>
+        <v>-0.05273305999018617</v>
       </c>
       <c r="C115" s="16" t="n">
-        <v>-0.05130103077915749</v>
+        <v>-0.051946717278759</v>
       </c>
       <c r="D115" s="16" t="n">
         <v>-0.09655190017960312</v>
@@ -3403,10 +3404,10 @@
         </is>
       </c>
       <c r="B116" s="15" t="n">
-        <v>0.1118308375366624</v>
+        <v>0.1111032252993529</v>
       </c>
       <c r="C116" s="15" t="n">
-        <v>0.08907652234311826</v>
+        <v>0.08656622608380825</v>
       </c>
       <c r="D116" s="15" t="n">
         <v>0.1264230081956648</v>
@@ -3431,10 +3432,10 @@
         </is>
       </c>
       <c r="B117" s="15" t="n">
-        <v>0.1269202867713231</v>
+        <v>0.1349358066749065</v>
       </c>
       <c r="C117" s="15" t="n">
-        <v>0.1126853249070437</v>
+        <v>0.1124895431472317</v>
       </c>
       <c r="D117" s="15" t="n">
         <v>0.1478031208157358</v>
@@ -3459,10 +3460,10 @@
         </is>
       </c>
       <c r="B118" s="15" t="n">
-        <v>0.01251692926503889</v>
+        <v>0.0124200540632704</v>
       </c>
       <c r="C118" s="15" t="n">
-        <v>0.01317538518677397</v>
+        <v>0.01290234322626493</v>
       </c>
       <c r="D118" s="15" t="n">
         <v>0.02140035205320401</v>
@@ -3487,10 +3488,10 @@
         </is>
       </c>
       <c r="B119" s="15" t="n">
-        <v>0.1139566103982528</v>
+        <v>0.1065648451868044</v>
       </c>
       <c r="C119" s="15" t="n">
-        <v>0.1070622544493802</v>
+        <v>0.104052987366096</v>
       </c>
       <c r="D119" s="15" t="n">
         <v>0.1620209006306683</v>
@@ -3515,10 +3516,10 @@
         </is>
       </c>
       <c r="B120" s="15" t="n">
-        <v>0.03383944566886155</v>
+        <v>0.02900567392670084</v>
       </c>
       <c r="C120" s="15" t="n">
-        <v>0.01854703766940346</v>
+        <v>0.01710420980395155</v>
       </c>
       <c r="D120" s="15" t="n">
         <v>0.009302151256766368</v>
@@ -3543,10 +3544,10 @@
         </is>
       </c>
       <c r="B121" s="16" t="n">
-        <v>-0.03919061189064443</v>
+        <v>-0.04201755965797337</v>
       </c>
       <c r="C121" s="16" t="n">
-        <v>-0.03170582642138753</v>
+        <v>-0.03012232362148337</v>
       </c>
       <c r="D121" s="16" t="n">
         <v>-0.05753190683091203</v>
@@ -3571,10 +3572,10 @@
         </is>
       </c>
       <c r="B122" s="15" t="n">
-        <v>0.05632987143950108</v>
+        <v>0.05000544459611334</v>
       </c>
       <c r="C122" s="15" t="n">
-        <v>0.03730730922141712</v>
+        <v>0.03393033233590725</v>
       </c>
       <c r="D122" s="15" t="n">
         <v>0.05662137159968883</v>
@@ -3599,10 +3600,10 @@
         </is>
       </c>
       <c r="B123" s="15" t="n">
-        <v>0.1262110614104763</v>
+        <v>0.1253344236111482</v>
       </c>
       <c r="C123" s="15" t="n">
-        <v>0.1159580804653128</v>
+        <v>0.1145157323299806</v>
       </c>
       <c r="D123" s="15" t="n">
         <v>0.1538755988480673</v>
@@ -3627,10 +3628,10 @@
         </is>
       </c>
       <c r="B124" s="16" t="n">
-        <v>-0.008727945545260574</v>
+        <v>-0.008039420706907552</v>
       </c>
       <c r="C124" s="16" t="n">
-        <v>-0.01259122048373185</v>
+        <v>-0.01318669525080307</v>
       </c>
       <c r="D124" s="16" t="n">
         <v>-0.05022954579430272</v>
@@ -3655,10 +3656,10 @@
         </is>
       </c>
       <c r="B125" s="15" t="n">
-        <v>0.02829687858024532</v>
+        <v>0.03264394136704962</v>
       </c>
       <c r="C125" s="15" t="n">
-        <v>0.004571604305015464</v>
+        <v>0.006856391500811965</v>
       </c>
       <c r="D125" s="16" t="n">
         <v>-0.039631970673079</v>
@@ -3683,10 +3684,10 @@
         </is>
       </c>
       <c r="B126" s="15" t="n">
-        <v>0.02195293417004107</v>
-      </c>
-      <c r="C126" s="15" t="n">
-        <v>0.001681102467018469</v>
+        <v>0.01338756301925037</v>
+      </c>
+      <c r="C126" s="16" t="n">
+        <v>-0.001159419764859448</v>
       </c>
       <c r="D126" s="16" t="n">
         <v>-0.02936818545736064</v>
@@ -3711,10 +3712,10 @@
         </is>
       </c>
       <c r="B127" s="16" t="n">
-        <v>-0.03954248384420811</v>
+        <v>-0.0420070021966109</v>
       </c>
       <c r="C127" s="16" t="n">
-        <v>-0.03491442095175401</v>
+        <v>-0.033666539372606</v>
       </c>
       <c r="D127" s="16" t="n">
         <v>-0.04273316852217701</v>
@@ -3739,10 +3740,10 @@
         </is>
       </c>
       <c r="B128" s="15" t="n">
-        <v>0.05937066622756193</v>
+        <v>0.05310702565041003</v>
       </c>
       <c r="C128" s="15" t="n">
-        <v>0.05568647828771756</v>
+        <v>0.05056127625763174</v>
       </c>
       <c r="D128" s="15" t="n">
         <v>0.1202591598579885</v>
@@ -3767,10 +3768,10 @@
         </is>
       </c>
       <c r="B129" s="16" t="n">
-        <v>-0.03920819945699428</v>
+        <v>-0.04402754534156673</v>
       </c>
       <c r="C129" s="16" t="n">
-        <v>-0.0298970722567915</v>
+        <v>-0.03228324907573554</v>
       </c>
       <c r="D129" s="16" t="n">
         <v>-0.03548647884703315</v>
@@ -3794,11 +3795,11 @@
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B130" s="15" t="n">
-        <v>0.01143383975941026</v>
+      <c r="B130" s="16" t="n">
+        <v>-0.002814978554845693</v>
       </c>
       <c r="C130" s="16" t="n">
-        <v>-0.008981655051958026</v>
+        <v>-0.01314262862641713</v>
       </c>
       <c r="D130" s="16" t="n">
         <v>-0.01127809447877726</v>
@@ -3823,10 +3824,10 @@
         </is>
       </c>
       <c r="B131" s="16" t="n">
-        <v>-0.04896142937237435</v>
+        <v>-0.03952128824422596</v>
       </c>
       <c r="C131" s="16" t="n">
-        <v>-0.04724185864380659</v>
+        <v>-0.0435716038747791</v>
       </c>
       <c r="D131" s="16" t="n">
         <v>-0.07455858091749135</v>
@@ -3851,10 +3852,10 @@
         </is>
       </c>
       <c r="B132" s="15" t="n">
-        <v>0.05975095309096257</v>
+        <v>0.03910806179183246</v>
       </c>
       <c r="C132" s="15" t="n">
-        <v>0.02171113494762245</v>
+        <v>0.01731152763095722</v>
       </c>
       <c r="D132" s="16" t="n">
         <v>-0.03380748124290922</v>
@@ -3879,10 +3880,10 @@
         </is>
       </c>
       <c r="B133" s="15" t="n">
-        <v>0.05214755528473369</v>
+        <v>0.03979349605369831</v>
       </c>
       <c r="C133" s="15" t="n">
-        <v>0.01911811052843904</v>
+        <v>0.0162835249684341</v>
       </c>
       <c r="D133" s="16" t="n">
         <v>-0.01503058922433043</v>
@@ -3907,10 +3908,10 @@
         </is>
       </c>
       <c r="B134" s="16" t="n">
-        <v>-0.01286171868699593</v>
+        <v>-0.01512565769251162</v>
       </c>
       <c r="C134" s="16" t="n">
-        <v>-0.006216466388790032</v>
+        <v>-0.003918405973913907</v>
       </c>
       <c r="D134" s="15" t="n">
         <v>0.001421239525864148</v>
@@ -3935,10 +3936,10 @@
         </is>
       </c>
       <c r="B135" s="15" t="n">
-        <v>0.1669990087457334</v>
+        <v>0.166545114027689</v>
       </c>
       <c r="C135" s="15" t="n">
-        <v>0.1547626790440761</v>
+        <v>0.1537640596603633</v>
       </c>
       <c r="D135" s="15" t="n">
         <v>0.2046404114382004</v>
@@ -3963,10 +3964,10 @@
         </is>
       </c>
       <c r="B136" s="15" t="n">
-        <v>0.089317582373887</v>
+        <v>0.09077487319247668</v>
       </c>
       <c r="C136" s="15" t="n">
-        <v>0.08490463642041401</v>
+        <v>0.08618069468885971</v>
       </c>
       <c r="D136" s="15" t="n">
         <v>0.1121372832146976</v>
@@ -3991,10 +3992,10 @@
         </is>
       </c>
       <c r="B137" s="15" t="n">
-        <v>0.04738794448678751</v>
+        <v>0.0438239756440888</v>
       </c>
       <c r="C137" s="15" t="n">
-        <v>0.04196596434885813</v>
+        <v>0.03877171054171558</v>
       </c>
       <c r="D137" s="15" t="n">
         <v>0.0404108750757084</v>
@@ -4019,10 +4020,10 @@
         </is>
       </c>
       <c r="B138" s="15" t="n">
-        <v>0.1304538644031215</v>
+        <v>0.1285851086141387</v>
       </c>
       <c r="C138" s="15" t="n">
-        <v>0.1063990571834419</v>
+        <v>0.1083786882744176</v>
       </c>
       <c r="D138" s="15" t="n">
         <v>0.1253149440594126</v>
@@ -4047,10 +4048,10 @@
         </is>
       </c>
       <c r="B139" s="15" t="n">
-        <v>0.09038495769507617</v>
+        <v>0.09337656105849067</v>
       </c>
       <c r="C139" s="15" t="n">
-        <v>0.07123005986374586</v>
+        <v>0.07693797180390916</v>
       </c>
       <c r="D139" s="15" t="n">
         <v>0.09941891513153278</v>
@@ -4075,10 +4076,10 @@
         </is>
       </c>
       <c r="B140" s="16" t="n">
-        <v>-0.06865372521563518</v>
+        <v>-0.0780670888665459</v>
       </c>
       <c r="C140" s="16" t="n">
-        <v>-0.07420076129851572</v>
+        <v>-0.07870962326308006</v>
       </c>
       <c r="D140" s="16" t="n">
         <v>-0.1153153654567373</v>
@@ -4103,10 +4104,10 @@
         </is>
       </c>
       <c r="B141" s="16" t="n">
-        <v>-0.01815341234433209</v>
+        <v>-0.01662836471020956</v>
       </c>
       <c r="C141" s="16" t="n">
-        <v>-0.02003305310419701</v>
+        <v>-0.01618772704309856</v>
       </c>
       <c r="D141" s="16" t="n">
         <v>-0.03016021812315839</v>
@@ -4131,10 +4132,10 @@
         </is>
       </c>
       <c r="B142" s="15" t="n">
-        <v>0.03560304676365855</v>
+        <v>0.05040178580008736</v>
       </c>
       <c r="C142" s="15" t="n">
-        <v>0.02706073591448588</v>
+        <v>0.03758905710757121</v>
       </c>
       <c r="D142" s="15" t="n">
         <v>0.02113175404862622</v>
@@ -4159,10 +4160,10 @@
         </is>
       </c>
       <c r="B143" s="16" t="n">
-        <v>-0.03120731775675945</v>
+        <v>-0.05133061165671194</v>
       </c>
       <c r="C143" s="16" t="n">
-        <v>-0.04542526094247867</v>
+        <v>-0.05557860855081776</v>
       </c>
       <c r="D143" s="16" t="n">
         <v>-0.09308439113318168</v>
@@ -4187,10 +4188,10 @@
         </is>
       </c>
       <c r="B144" s="16" t="n">
-        <v>-0.1130775796200464</v>
+        <v>-0.08695476094268806</v>
       </c>
       <c r="C144" s="16" t="n">
-        <v>-0.06676742193858798</v>
+        <v>-0.05928830177989141</v>
       </c>
       <c r="D144" s="16" t="n">
         <v>-0.04096163768438366</v>

</xml_diff>